<commit_message>
Update .env.example with Gmail configuration for agent activation; adjust Playwright retries to 0; update yarn.lock to use npm registry; remove outdated HRMS testing documentation files.
</commit_message>
<xml_diff>
--- a/TestFiles-prod-sanity/AdvanceAndAdjustment/[MLB]AdvanceStatement-AA [Recovery].xlsx
+++ b/TestFiles-prod-sanity/AdvanceAndAdjustment/[MLB]AdvanceStatement-AA [Recovery].xlsx
@@ -97,7 +97,7 @@
     <t>IL</t>
   </si>
   <si>
-    <t>test-aetna-aca-test-advance-month-july-21</t>
+    <t>test-aetna-aca-advance-july-21</t>
   </si>
   <si>
     <t>Y</t>
@@ -174,9 +174,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -527,571 +526,571 @@
   <dimension ref="A1:Z8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.14785714285714" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.433571428571426" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.147857142857141" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.576428571428572" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.576428571428572" style="2" customWidth="1"/>
-    <col min="6" max="6" width="13.576428571428572" style="1" customWidth="1"/>
-    <col min="7" max="7" width="22.719285714285714" style="1" customWidth="1"/>
-    <col min="8" max="8" width="19.433571428571426" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.862142857142857" style="3" customWidth="1"/>
-    <col min="10" max="10" width="13.576428571428572" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.576428571428572" style="3" customWidth="1"/>
-    <col min="12" max="12" width="13.576428571428572" style="2" customWidth="1"/>
-    <col min="13" max="13" width="13.576428571428572" style="4" customWidth="1"/>
-    <col min="14" max="14" width="13.576428571428572" style="2" customWidth="1"/>
-    <col min="15" max="15" width="17.14785714285714" style="2" customWidth="1"/>
-    <col min="16" max="16" width="20.14785714285714" style="1" customWidth="1"/>
-    <col min="17" max="17" width="13.576428571428572" style="3" customWidth="1"/>
-    <col min="18" max="19" width="13.576428571428572" style="1" customWidth="1"/>
-    <col min="20" max="20" width="13.576428571428572" style="2" customWidth="1"/>
-    <col min="21" max="26" width="13.576428571428572" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.14785714285714" customWidth="1"/>
+    <col min="2" max="2" width="18.433571428571426" customWidth="1"/>
+    <col min="3" max="3" width="14.147857142857141" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.576428571428572" customWidth="1"/>
+    <col min="5" max="5" width="13.576428571428572" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.576428571428572" customWidth="1"/>
+    <col min="7" max="7" width="22.719285714285714" customWidth="1"/>
+    <col min="8" max="8" width="19.433571428571426" customWidth="1"/>
+    <col min="9" max="9" width="20.862142857142857" style="2" customWidth="1"/>
+    <col min="10" max="10" width="13.576428571428572" customWidth="1"/>
+    <col min="11" max="11" width="13.576428571428572" style="2" customWidth="1"/>
+    <col min="12" max="12" width="13.576428571428572" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.576428571428572" style="3" customWidth="1"/>
+    <col min="14" max="14" width="13.576428571428572" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.14785714285714" style="1" customWidth="1"/>
+    <col min="16" max="16" width="20.14785714285714" customWidth="1"/>
+    <col min="17" max="17" width="13.576428571428572" style="2" customWidth="1"/>
+    <col min="18" max="19" width="13.576428571428572" customWidth="1"/>
+    <col min="20" max="20" width="13.576428571428572" style="1" customWidth="1"/>
+    <col min="21" max="26" width="13.576428571428572" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="T1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-      <c r="W1" s="9"/>
-      <c r="X1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="Z1" s="9"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
     </row>
     <row r="2" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="11">
         <v>600011</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="13">
-        <v>1</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="12">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="14">
-        <v>44197</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="H2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="13">
+        <v>44197</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K2" s="14">
-        <v>44197</v>
-      </c>
-      <c r="L2" s="13">
-        <v>1</v>
-      </c>
-      <c r="M2" s="15">
+      <c r="K2" s="13">
+        <v>44197</v>
+      </c>
+      <c r="L2" s="12">
+        <v>1</v>
+      </c>
+      <c r="M2" s="14">
         <v>78.9</v>
       </c>
-      <c r="N2" s="13">
+      <c r="N2" s="12">
         <v>0</v>
       </c>
-      <c r="O2" s="13">
-        <v>25</v>
-      </c>
-      <c r="P2" s="5" t="s">
+      <c r="O2" s="12">
+        <v>25</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" s="14">
+      <c r="Q2" s="13">
         <v>44198</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="R2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="S2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T2" s="13">
+      <c r="T2" s="12">
         <v>789</v>
       </c>
-      <c r="U2" s="9"/>
-      <c r="V2" s="9"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="8"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+      <c r="Y2" s="8"/>
+      <c r="Z2" s="8"/>
     </row>
     <row r="3" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="11">
         <v>600011</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="13">
-        <v>1</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="E3" s="12">
+        <v>1</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="14">
-        <v>44197</v>
-      </c>
-      <c r="J3" s="5" t="s">
+      <c r="H3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="13">
+        <v>44197</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="14">
-        <v>44197</v>
-      </c>
-      <c r="L3" s="13">
-        <v>1</v>
-      </c>
-      <c r="M3" s="15">
+      <c r="K3" s="13">
+        <v>44197</v>
+      </c>
+      <c r="L3" s="12">
+        <v>1</v>
+      </c>
+      <c r="M3" s="14">
         <v>78.9</v>
       </c>
-      <c r="N3" s="13">
+      <c r="N3" s="12">
         <v>0</v>
       </c>
-      <c r="O3" s="13">
-        <v>25</v>
-      </c>
-      <c r="P3" s="5" t="s">
+      <c r="O3" s="12">
+        <v>25</v>
+      </c>
+      <c r="P3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q3" s="14">
+      <c r="Q3" s="13">
         <v>44228</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="R3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="S3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T3" s="13">
+      <c r="T3" s="12">
         <v>789</v>
       </c>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
-      <c r="W3" s="9"/>
-      <c r="X3" s="9"/>
-      <c r="Y3" s="9"/>
-      <c r="Z3" s="9"/>
+      <c r="U3" s="8"/>
+      <c r="V3" s="8"/>
+      <c r="W3" s="8"/>
+      <c r="X3" s="8"/>
+      <c r="Y3" s="8"/>
+      <c r="Z3" s="8"/>
     </row>
     <row r="4" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="11">
         <v>600011</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="13">
-        <v>1</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="E4" s="12">
+        <v>1</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" s="14">
-        <v>44197</v>
-      </c>
-      <c r="J4" s="5" t="s">
+      <c r="H4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="13">
+        <v>44197</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="14">
-        <v>44197</v>
-      </c>
-      <c r="L4" s="13">
-        <v>1</v>
-      </c>
-      <c r="M4" s="15">
+      <c r="K4" s="13">
+        <v>44197</v>
+      </c>
+      <c r="L4" s="12">
+        <v>1</v>
+      </c>
+      <c r="M4" s="14">
         <v>78.9</v>
       </c>
-      <c r="N4" s="13">
+      <c r="N4" s="12">
         <v>0</v>
       </c>
-      <c r="O4" s="13">
-        <v>25</v>
-      </c>
-      <c r="P4" s="5" t="s">
+      <c r="O4" s="12">
+        <v>25</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q4" s="14">
+      <c r="Q4" s="13">
         <v>44256</v>
       </c>
-      <c r="R4" s="5" t="s">
+      <c r="R4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="S4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T4" s="13">
+      <c r="T4" s="12">
         <v>789</v>
       </c>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
-      <c r="W4" s="9"/>
-      <c r="X4" s="9"/>
-      <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
+      <c r="U4" s="8"/>
+      <c r="V4" s="8"/>
+      <c r="W4" s="8"/>
+      <c r="X4" s="8"/>
+      <c r="Y4" s="8"/>
+      <c r="Z4" s="8"/>
     </row>
     <row r="5" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="11">
         <v>600011</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="13">
-        <v>1</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="12">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" s="14">
-        <v>44197</v>
-      </c>
-      <c r="J5" s="5" t="s">
+      <c r="H5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="13">
+        <v>44197</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K5" s="14">
-        <v>44197</v>
-      </c>
-      <c r="L5" s="13">
-        <v>1</v>
-      </c>
-      <c r="M5" s="15">
+      <c r="K5" s="13">
+        <v>44197</v>
+      </c>
+      <c r="L5" s="12">
+        <v>1</v>
+      </c>
+      <c r="M5" s="14">
         <v>78.9</v>
       </c>
-      <c r="N5" s="13">
+      <c r="N5" s="12">
         <v>0</v>
       </c>
-      <c r="O5" s="13">
-        <v>25</v>
-      </c>
-      <c r="P5" s="5" t="s">
+      <c r="O5" s="12">
+        <v>25</v>
+      </c>
+      <c r="P5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q5" s="14">
+      <c r="Q5" s="13">
         <v>44287</v>
       </c>
-      <c r="R5" s="5" t="s">
+      <c r="R5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S5" s="5" t="s">
+      <c r="S5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T5" s="13">
+      <c r="T5" s="12">
         <v>789</v>
       </c>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
-      <c r="W5" s="9"/>
-      <c r="X5" s="9"/>
-      <c r="Y5" s="9"/>
-      <c r="Z5" s="9"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="8"/>
+      <c r="W5" s="8"/>
+      <c r="X5" s="8"/>
+      <c r="Y5" s="8"/>
+      <c r="Z5" s="8"/>
     </row>
     <row r="6" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="11">
         <v>600011</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="13">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="E6" s="12">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" s="14">
-        <v>44197</v>
-      </c>
-      <c r="J6" s="5" t="s">
+      <c r="H6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="13">
+        <v>44197</v>
+      </c>
+      <c r="J6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K6" s="14">
-        <v>44197</v>
-      </c>
-      <c r="L6" s="13">
-        <v>1</v>
-      </c>
-      <c r="M6" s="15">
+      <c r="K6" s="13">
+        <v>44197</v>
+      </c>
+      <c r="L6" s="12">
+        <v>1</v>
+      </c>
+      <c r="M6" s="14">
         <v>78.9</v>
       </c>
-      <c r="N6" s="13">
+      <c r="N6" s="12">
         <v>0</v>
       </c>
-      <c r="O6" s="13">
-        <v>25</v>
-      </c>
-      <c r="P6" s="5" t="s">
+      <c r="O6" s="12">
+        <v>25</v>
+      </c>
+      <c r="P6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q6" s="14">
+      <c r="Q6" s="13">
         <v>44317</v>
       </c>
-      <c r="R6" s="5" t="s">
+      <c r="R6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S6" s="5" t="s">
+      <c r="S6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T6" s="13">
+      <c r="T6" s="12">
         <v>789</v>
       </c>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
-      <c r="Y6" s="9"/>
-      <c r="Z6" s="9"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="8"/>
+      <c r="W6" s="8"/>
+      <c r="X6" s="8"/>
+      <c r="Y6" s="8"/>
+      <c r="Z6" s="8"/>
     </row>
     <row r="7" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="11">
         <v>600011</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="13">
-        <v>1</v>
-      </c>
-      <c r="F7" s="5" t="s">
+      <c r="E7" s="12">
+        <v>1</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I7" s="14">
-        <v>44197</v>
-      </c>
-      <c r="J7" s="5" t="s">
+      <c r="H7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="13">
+        <v>44197</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K7" s="14">
-        <v>44197</v>
-      </c>
-      <c r="L7" s="13">
-        <v>1</v>
-      </c>
-      <c r="M7" s="15">
+      <c r="K7" s="13">
+        <v>44197</v>
+      </c>
+      <c r="L7" s="12">
+        <v>1</v>
+      </c>
+      <c r="M7" s="14">
         <v>78.9</v>
       </c>
-      <c r="N7" s="13">
+      <c r="N7" s="12">
         <v>0</v>
       </c>
-      <c r="O7" s="13">
-        <v>25</v>
-      </c>
-      <c r="P7" s="5" t="s">
+      <c r="O7" s="12">
+        <v>25</v>
+      </c>
+      <c r="P7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q7" s="14">
+      <c r="Q7" s="13">
         <v>44348</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="R7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S7" s="5" t="s">
+      <c r="S7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T7" s="13">
+      <c r="T7" s="12">
         <v>789</v>
       </c>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9"/>
-      <c r="Y7" s="9"/>
-      <c r="Z7" s="9"/>
+      <c r="U7" s="8"/>
+      <c r="V7" s="8"/>
+      <c r="W7" s="8"/>
+      <c r="X7" s="8"/>
+      <c r="Y7" s="8"/>
+      <c r="Z7" s="8"/>
     </row>
     <row r="8" ht="19.5" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="11">
         <v>600011</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="13">
-        <v>1</v>
-      </c>
-      <c r="F8" s="5" t="s">
+      <c r="E8" s="12">
+        <v>1</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I8" s="14">
-        <v>44197</v>
-      </c>
-      <c r="J8" s="5" t="s">
+      <c r="H8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="13">
+        <v>44197</v>
+      </c>
+      <c r="J8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K8" s="14">
-        <v>44197</v>
-      </c>
-      <c r="L8" s="13">
-        <v>1</v>
-      </c>
-      <c r="M8" s="15">
+      <c r="K8" s="13">
+        <v>44197</v>
+      </c>
+      <c r="L8" s="12">
+        <v>1</v>
+      </c>
+      <c r="M8" s="14">
         <v>78.9</v>
       </c>
-      <c r="N8" s="13">
+      <c r="N8" s="12">
         <v>0</v>
       </c>
-      <c r="O8" s="13">
-        <v>25</v>
-      </c>
-      <c r="P8" s="5" t="s">
+      <c r="O8" s="12">
+        <v>25</v>
+      </c>
+      <c r="P8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q8" s="14">
+      <c r="Q8" s="13">
         <v>44378</v>
       </c>
-      <c r="R8" s="5" t="s">
+      <c r="R8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S8" s="5" t="s">
+      <c r="S8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="T8" s="13">
+      <c r="T8" s="12">
         <v>789</v>
       </c>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="8"/>
+      <c r="W8" s="8"/>
+      <c r="X8" s="8"/>
+      <c r="Y8" s="8"/>
+      <c r="Z8" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>